<commit_message>
sửa giao diện admin
</commit_message>
<xml_diff>
--- a/VNUFLearning/wwwroot/templates/MauImportCauHoi.xlsx
+++ b/VNUFLearning/wwwroot/templates/MauImportCauHoi.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\KLTN1\VNUFLearning\VNUFLearning\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\KLTN1\VNUFLearning\VNUFLearning\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90F8D287-BD7B-46DD-85D1-E7F2133D4E1A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48E6ACDE-57EB-48E1-A5D0-4792FA0DDF86}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{80BAE5D0-5909-48F2-A6F9-137997754082}"/>
   </bookViews>
@@ -31,10 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t>SubjectId</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>QuestionType</t>
   </si>
@@ -423,17 +420,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAE9B530-9C3A-4399-865B-C83D921D63CF}">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="16.33203125" customWidth="1"/>
     <col min="3" max="3" width="21.109375" customWidth="1"/>
-    <col min="8" max="8" width="13.88671875" customWidth="1"/>
+    <col min="7" max="7" width="14.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -451,17 +448,13 @@
         <v>4</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H2" s="2"/>
       <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>